<commit_message>
Robustness fixes from 5 unseen tenders: 2-page PDF reading, continuation pages, quantities parsed and checked against the PDF, kind-of-work rule, unique line keys, rebar and general metal works items, unit choice on conflicts
</commit_message>
<xml_diff>
--- a/Price list - steel and metal works.xlsx
+++ b/Price list - steel and metal works.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Downloads\OnTap hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A109D8EB-E3B8-4F59-9472-6ABCE147DC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1940CF-538A-4A45-84C5-C8DE69C9D8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="291">
   <si>
     <t>Price list - steel structures, metal works and construction works (Cairo, 2026)</t>
   </si>
@@ -301,6 +301,21 @@
     <t>Flat bar 6 m</t>
   </si>
   <si>
+    <t>MW-07</t>
+  </si>
+  <si>
+    <t>أعمال حدادة عامة وحديد كريتال توريد وتصنيع وتركيب ودهان</t>
+  </si>
+  <si>
+    <t>General metal works and crittall steel: supply, fabricate, install and paint</t>
+  </si>
+  <si>
+    <t>Medium angles 60-100 mm</t>
+  </si>
+  <si>
+    <t>New item (Sep 2026): built from existing rates - please check</t>
+  </si>
+  <si>
     <t>CW-01</t>
   </si>
   <si>
@@ -538,6 +553,18 @@
     <t>no. / عدد</t>
   </si>
   <si>
+    <t>CW-26</t>
+  </si>
+  <si>
+    <t>توريد وتقطيع وتشكيل وتركيب حديد التسليح</t>
+  </si>
+  <si>
+    <t>Rebar, supply, cut, bend and fix</t>
+  </si>
+  <si>
+    <t>New item (Sep 2026): rebar + fixing from the reviewer's rates - please check</t>
+  </si>
+  <si>
     <t>Cairo prices, including tax, excluding transport. Yellow = estimate, please check. No overhead or profit here.</t>
   </si>
   <si>
@@ -575,9 +602,6 @@
   </si>
   <si>
     <t>زوايا ثقيلة من 120 إلى 200 مم</t>
-  </si>
-  <si>
-    <t>Medium angles 60-100 mm</t>
   </si>
   <si>
     <t>زوايا متوسطة من 60 إلى 100 مم</t>
@@ -991,7 +1015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1032,10 +1056,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
@@ -1443,7 +1470,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R38"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1838,32 +1865,32 @@
         <v>1000</v>
       </c>
       <c r="H8" s="10">
-        <f t="shared" ref="H8:H13" si="0">ROUND(VLOOKUP($F8,Materials,3,FALSE)*(1+IF($E8="Structure",WasteStructure,WasteMetal)),0)</f>
+        <f t="shared" ref="H8:H14" si="0">ROUND(VLOOKUP($F8,Materials,3,FALSE)*(1+IF($E8="Structure",WasteStructure,WasteMetal)),0)</f>
         <v>56100</v>
       </c>
       <c r="I8" s="10">
-        <f t="shared" ref="I8:I13" si="1">ROUND(VLOOKUP($F8,Materials,3,FALSE)*Consumables,0)</f>
+        <f t="shared" ref="I8:I14" si="1">ROUND(VLOOKUP($F8,Materials,3,FALSE)*Consumables,0)</f>
         <v>1530</v>
       </c>
       <c r="J8" s="10">
-        <f t="shared" ref="J8:J13" si="2">IF($E8="Structure",FabStructure,FabMetal)</f>
+        <f t="shared" ref="J8:J14" si="2">IF($E8="Structure",FabStructure,FabMetal)</f>
         <v>30000</v>
       </c>
       <c r="K8" s="10">
-        <f t="shared" ref="K8:K13" si="3">Paint</f>
+        <f t="shared" ref="K8:K14" si="3">Paint</f>
         <v>2500</v>
       </c>
       <c r="L8" s="10">
-        <f t="shared" ref="L8:L13" si="4">Transport</f>
+        <f t="shared" ref="L8:L14" si="4">Transport</f>
         <v>1200</v>
       </c>
       <c r="M8" s="11">
-        <f t="shared" ref="M8:M13" si="5">SUM(H8:L8)</f>
+        <f t="shared" ref="M8:M14" si="5">SUM(H8:L8)</f>
         <v>91330</v>
       </c>
       <c r="N8" s="10"/>
       <c r="O8" s="12">
-        <f t="shared" ref="O8:O13" si="6">ROUND(G8/1000*M8,0)</f>
+        <f t="shared" ref="O8:O14" si="6">ROUND(G8/1000*M8,0)</f>
         <v>91330</v>
       </c>
       <c r="P8" s="9"/>
@@ -2153,8 +2180,8 @@
       <c r="Q13" s="10"/>
       <c r="R13" s="9"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="13" t="s">
         <v>81</v>
       </c>
       <c r="B14" s="8" t="s">
@@ -2164,48 +2191,67 @@
         <v>83</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="G14" s="7">
+        <v>1000</v>
+      </c>
+      <c r="H14" s="10">
+        <f t="shared" si="0"/>
+        <v>52800</v>
+      </c>
+      <c r="I14" s="10">
+        <f t="shared" si="1"/>
+        <v>1440</v>
+      </c>
+      <c r="J14" s="10">
+        <f t="shared" si="2"/>
+        <v>30000</v>
+      </c>
+      <c r="K14" s="10">
+        <f t="shared" si="3"/>
+        <v>2500</v>
+      </c>
+      <c r="L14" s="10">
+        <f t="shared" si="4"/>
+        <v>1200</v>
+      </c>
+      <c r="M14" s="11">
+        <f t="shared" si="5"/>
+        <v>87940</v>
+      </c>
+      <c r="N14" s="10"/>
+      <c r="O14" s="14">
+        <f t="shared" si="6"/>
+        <v>87940</v>
+      </c>
+      <c r="P14" s="15" t="s">
         <v>85</v>
-      </c>
-      <c r="F14" s="9"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="10">
-        <f>Construction!$E$36</f>
-        <v>130</v>
-      </c>
-      <c r="O14" s="12">
-        <f t="shared" ref="O14:O38" si="7">N14</f>
-        <v>130</v>
-      </c>
-      <c r="P14" s="9" t="s">
-        <v>86</v>
       </c>
       <c r="Q14" s="10"/>
       <c r="R14" s="9"/>
     </row>
-    <row r="15" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="D15" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>84</v>
-      </c>
       <c r="E15" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="7"/>
@@ -2216,34 +2262,34 @@
       <c r="L15" s="10"/>
       <c r="M15" s="11"/>
       <c r="N15" s="10">
-        <f>Construction!$E$37</f>
-        <v>480</v>
+        <f>Construction!$E$36</f>
+        <v>130</v>
       </c>
       <c r="O15" s="12">
-        <f t="shared" si="7"/>
-        <v>480</v>
+        <f t="shared" ref="O15:O40" si="7">N15</f>
+        <v>130</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q15" s="10"/>
       <c r="R15" s="9"/>
     </row>
     <row r="16" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>85</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="7"/>
@@ -2254,34 +2300,34 @@
       <c r="L16" s="10"/>
       <c r="M16" s="11"/>
       <c r="N16" s="10">
-        <f>Construction!$E$38</f>
-        <v>120</v>
+        <f>Construction!$E$37</f>
+        <v>480</v>
       </c>
       <c r="O16" s="12">
         <f t="shared" si="7"/>
-        <v>120</v>
+        <v>480</v>
       </c>
       <c r="P16" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q16" s="10"/>
       <c r="R16" s="9"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="7"/>
@@ -2292,34 +2338,34 @@
       <c r="L17" s="10"/>
       <c r="M17" s="11"/>
       <c r="N17" s="10">
-        <f>Construction!$L$20</f>
-        <v>3000</v>
+        <f>Construction!$E$38</f>
+        <v>120</v>
       </c>
       <c r="O17" s="12">
         <f t="shared" si="7"/>
-        <v>3000</v>
+        <v>120</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q17" s="10"/>
       <c r="R17" s="9"/>
     </row>
-    <row r="18" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="7"/>
@@ -2330,34 +2376,34 @@
       <c r="L18" s="10"/>
       <c r="M18" s="11"/>
       <c r="N18" s="10">
-        <f>Construction!$L$21</f>
-        <v>8100</v>
+        <f>Construction!$L$20</f>
+        <v>3000</v>
       </c>
       <c r="O18" s="12">
         <f t="shared" si="7"/>
-        <v>8100</v>
+        <v>3000</v>
       </c>
       <c r="P18" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q18" s="10"/>
       <c r="R18" s="9"/>
     </row>
     <row r="19" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="7"/>
@@ -2368,34 +2414,34 @@
       <c r="L19" s="10"/>
       <c r="M19" s="11"/>
       <c r="N19" s="10">
-        <f>Construction!$L$22</f>
-        <v>4500</v>
+        <f>Construction!$L$21</f>
+        <v>8100</v>
       </c>
       <c r="O19" s="12">
         <f t="shared" si="7"/>
-        <v>4500</v>
+        <v>8100</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q19" s="10"/>
       <c r="R19" s="9"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="7"/>
@@ -2406,34 +2452,34 @@
       <c r="L20" s="10"/>
       <c r="M20" s="11"/>
       <c r="N20" s="10">
-        <f>Construction!$L$23</f>
-        <v>9635</v>
+        <f>Construction!$L$22</f>
+        <v>4500</v>
       </c>
       <c r="O20" s="12">
         <f t="shared" si="7"/>
-        <v>9635</v>
+        <v>4500</v>
       </c>
       <c r="P20" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q20" s="10"/>
       <c r="R20" s="9"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="7"/>
@@ -2444,34 +2490,34 @@
       <c r="L21" s="10"/>
       <c r="M21" s="11"/>
       <c r="N21" s="10">
-        <f>Construction!$L$24</f>
-        <v>12500</v>
+        <f>Construction!$L$23</f>
+        <v>9635</v>
       </c>
       <c r="O21" s="12">
         <f t="shared" si="7"/>
-        <v>12500</v>
+        <v>9635</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q21" s="10"/>
       <c r="R21" s="9"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="7"/>
@@ -2482,34 +2528,34 @@
       <c r="L22" s="10"/>
       <c r="M22" s="11"/>
       <c r="N22" s="10">
-        <f>Construction!$L$25</f>
-        <v>9300</v>
+        <f>Construction!$L$24</f>
+        <v>12500</v>
       </c>
       <c r="O22" s="12">
         <f t="shared" si="7"/>
-        <v>9300</v>
+        <v>12500</v>
       </c>
       <c r="P22" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q22" s="10"/>
       <c r="R22" s="9"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="7"/>
@@ -2520,34 +2566,34 @@
       <c r="L23" s="10"/>
       <c r="M23" s="11"/>
       <c r="N23" s="10">
-        <f>Construction!$L$26</f>
-        <v>9500</v>
+        <f>Construction!$L$25</f>
+        <v>9300</v>
       </c>
       <c r="O23" s="12">
         <f t="shared" si="7"/>
-        <v>9500</v>
+        <v>9300</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q23" s="10"/>
       <c r="R23" s="9"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="7"/>
@@ -2558,34 +2604,34 @@
       <c r="L24" s="10"/>
       <c r="M24" s="11"/>
       <c r="N24" s="10">
-        <f>Construction!$L$27</f>
-        <v>9550</v>
+        <f>Construction!$L$26</f>
+        <v>9500</v>
       </c>
       <c r="O24" s="12">
         <f t="shared" si="7"/>
-        <v>9550</v>
+        <v>9500</v>
       </c>
       <c r="P24" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q24" s="10"/>
       <c r="R24" s="9"/>
     </row>
-    <row r="25" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="7"/>
@@ -2596,34 +2642,34 @@
       <c r="L25" s="10"/>
       <c r="M25" s="11"/>
       <c r="N25" s="10">
-        <f>Construction!$K$30</f>
-        <v>600.125</v>
+        <f>Construction!$L$27</f>
+        <v>9550</v>
       </c>
       <c r="O25" s="12">
         <f t="shared" si="7"/>
-        <v>600.125</v>
+        <v>9550</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="9"/>
     </row>
     <row r="26" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="7"/>
@@ -2634,34 +2680,34 @@
       <c r="L26" s="10"/>
       <c r="M26" s="11"/>
       <c r="N26" s="10">
-        <f>Construction!$K$31</f>
-        <v>320.9425</v>
+        <f>Construction!$K$30</f>
+        <v>600.125</v>
       </c>
       <c r="O26" s="12">
         <f t="shared" si="7"/>
-        <v>320.9425</v>
+        <v>600.125</v>
       </c>
       <c r="P26" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q26" s="10"/>
       <c r="R26" s="9"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="7"/>
@@ -2672,34 +2718,34 @@
       <c r="L27" s="10"/>
       <c r="M27" s="11"/>
       <c r="N27" s="10">
-        <f>Construction!$K$32</f>
-        <v>1001</v>
+        <f>Construction!$K$31</f>
+        <v>320.9425</v>
       </c>
       <c r="O27" s="12">
         <f t="shared" si="7"/>
-        <v>1001</v>
+        <v>320.9425</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="9"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="7"/>
@@ -2710,34 +2756,34 @@
       <c r="L28" s="10"/>
       <c r="M28" s="11"/>
       <c r="N28" s="10">
-        <f>Construction!$K$33</f>
-        <v>500.08</v>
+        <f>Construction!$K$32</f>
+        <v>1001</v>
       </c>
       <c r="O28" s="12">
         <f t="shared" si="7"/>
-        <v>500.08</v>
+        <v>1001</v>
       </c>
       <c r="P28" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q28" s="10"/>
       <c r="R28" s="9"/>
     </row>
-    <row r="29" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="7"/>
@@ -2748,34 +2794,34 @@
       <c r="L29" s="10"/>
       <c r="M29" s="11"/>
       <c r="N29" s="10">
-        <f>Construction!$E$39</f>
-        <v>330</v>
+        <f>Construction!$K$33</f>
+        <v>500.08</v>
       </c>
       <c r="O29" s="12">
         <f t="shared" si="7"/>
-        <v>330</v>
+        <v>500.08</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q29" s="10"/>
       <c r="R29" s="9"/>
     </row>
     <row r="30" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="7"/>
@@ -2786,34 +2832,34 @@
       <c r="L30" s="10"/>
       <c r="M30" s="11"/>
       <c r="N30" s="10">
-        <f>Construction!$E$40</f>
-        <v>350</v>
+        <f>Construction!$E$39</f>
+        <v>330</v>
       </c>
       <c r="O30" s="12">
         <f t="shared" si="7"/>
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="P30" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q30" s="10"/>
       <c r="R30" s="9"/>
     </row>
     <row r="31" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="7"/>
@@ -2824,34 +2870,34 @@
       <c r="L31" s="10"/>
       <c r="M31" s="11"/>
       <c r="N31" s="10">
-        <f>Construction!$E$41</f>
-        <v>260</v>
+        <f>Construction!$E$40</f>
+        <v>350</v>
       </c>
       <c r="O31" s="12">
         <f t="shared" si="7"/>
-        <v>260</v>
+        <v>350</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="9"/>
     </row>
     <row r="32" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="7"/>
@@ -2862,34 +2908,34 @@
       <c r="L32" s="10"/>
       <c r="M32" s="11"/>
       <c r="N32" s="10">
-        <f>Construction!$E$42</f>
-        <v>250</v>
+        <f>Construction!$E$41</f>
+        <v>260</v>
       </c>
       <c r="O32" s="12">
         <f t="shared" si="7"/>
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="P32" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q32" s="10"/>
       <c r="R32" s="9"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="7"/>
@@ -2900,34 +2946,34 @@
       <c r="L33" s="10"/>
       <c r="M33" s="11"/>
       <c r="N33" s="10">
-        <f>Construction!$E$43</f>
-        <v>185</v>
+        <f>Construction!$E$42</f>
+        <v>250</v>
       </c>
       <c r="O33" s="12">
         <f t="shared" si="7"/>
-        <v>185</v>
+        <v>250</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q33" s="10"/>
       <c r="R33" s="9"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="7"/>
@@ -2938,34 +2984,34 @@
       <c r="L34" s="10"/>
       <c r="M34" s="11"/>
       <c r="N34" s="10">
-        <f>Construction!$E$44</f>
-        <v>270</v>
+        <f>Construction!$E$43</f>
+        <v>185</v>
       </c>
       <c r="O34" s="12">
         <f t="shared" si="7"/>
-        <v>270</v>
+        <v>185</v>
       </c>
       <c r="P34" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q34" s="10"/>
       <c r="R34" s="9"/>
     </row>
-    <row r="35" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="7"/>
@@ -2976,34 +3022,34 @@
       <c r="L35" s="10"/>
       <c r="M35" s="11"/>
       <c r="N35" s="10">
-        <f>Construction!$E$45</f>
-        <v>4200</v>
+        <f>Construction!$E$44</f>
+        <v>270</v>
       </c>
       <c r="O35" s="12">
         <f t="shared" si="7"/>
-        <v>4200</v>
+        <v>270</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="9"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="7"/>
@@ -3014,34 +3060,34 @@
       <c r="L36" s="10"/>
       <c r="M36" s="11"/>
       <c r="N36" s="10">
-        <f>Construction!$E$46</f>
-        <v>300</v>
+        <f>Construction!$E$45</f>
+        <v>4200</v>
       </c>
       <c r="O36" s="12">
         <f t="shared" si="7"/>
-        <v>300</v>
+        <v>4200</v>
       </c>
       <c r="P36" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q36" s="10"/>
       <c r="R36" s="9"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="7"/>
@@ -3052,34 +3098,34 @@
       <c r="L37" s="10"/>
       <c r="M37" s="11"/>
       <c r="N37" s="10">
-        <f>Construction!$E$47</f>
-        <v>2300</v>
+        <f>Construction!$E$46</f>
+        <v>300</v>
       </c>
       <c r="O37" s="12">
         <f t="shared" si="7"/>
-        <v>2300</v>
+        <v>300</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="9"/>
     </row>
-    <row r="38" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>159</v>
+        <v>43</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="7"/>
@@ -3090,18 +3136,94 @@
       <c r="L38" s="10"/>
       <c r="M38" s="11"/>
       <c r="N38" s="10">
+        <f>Construction!$E$47</f>
+        <v>2300</v>
+      </c>
+      <c r="O38" s="12">
+        <f t="shared" si="7"/>
+        <v>2300</v>
+      </c>
+      <c r="P38" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q38" s="10"/>
+      <c r="R38" s="9"/>
+    </row>
+    <row r="39" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+      <c r="A39" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F39" s="9"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="11"/>
+      <c r="N39" s="10">
         <f>Construction!$E$48</f>
         <v>750000</v>
       </c>
-      <c r="O38" s="12">
+      <c r="O39" s="12">
         <f t="shared" si="7"/>
         <v>750000</v>
       </c>
-      <c r="P38" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q38" s="10"/>
-      <c r="R38" s="9"/>
+      <c r="P39" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q39" s="10"/>
+      <c r="R39" s="9"/>
+    </row>
+    <row r="40" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F40" s="9"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="11"/>
+      <c r="N40" s="10">
+        <f>Construction!$E$49</f>
+        <v>41000</v>
+      </c>
+      <c r="O40" s="14">
+        <f t="shared" si="7"/>
+        <v>41000</v>
+      </c>
+      <c r="P40" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3121,29 +3243,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
+      <c r="A1" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
@@ -3151,13 +3273,13 @@
         <v>35</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="C4" s="10">
         <v>57600</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E4" s="7">
         <v>7</v>
@@ -3168,13 +3290,13 @@
         <v>39</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="C5" s="10">
         <v>51000</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E5" s="7">
         <v>7</v>
@@ -3182,16 +3304,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="C6" s="10">
         <v>48000</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E6" s="7">
         <v>7</v>
@@ -3199,16 +3321,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="C7" s="10">
         <v>54000</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E7" s="7">
         <v>7</v>
@@ -3216,16 +3338,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>173</v>
+        <v>84</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C8" s="10">
         <v>48000</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E8" s="7">
         <v>8</v>
@@ -3233,16 +3355,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C9" s="10">
         <v>45000</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E9" s="7">
         <v>8</v>
@@ -3253,13 +3375,13 @@
         <v>80</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="C10" s="10">
         <v>43000</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E10" s="7">
         <v>8</v>
@@ -3270,13 +3392,13 @@
         <v>73</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C11" s="10">
         <v>54000</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E11" s="7">
         <v>8</v>
@@ -3287,13 +3409,13 @@
         <v>48</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C12" s="10">
         <v>46000</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E12" s="7">
         <v>134</v>
@@ -3304,13 +3426,13 @@
         <v>63</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="C13" s="10">
         <v>52000</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="E13" s="7">
         <v>134</v>
@@ -3321,28 +3443,28 @@
         <v>68</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C14" s="10">
         <v>46700</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="E14" s="7"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>15</v>
@@ -3350,189 +3472,189 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="C17" s="10">
         <v>15000</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="C18" s="17">
+        <v>198</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="C18" s="18">
         <v>30000</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="C19" s="17">
+        <v>201</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="C19" s="18">
         <v>2500</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15" t="s">
-        <v>195</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="C20" s="18">
+        <v>203</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C20" s="19">
         <v>0.05</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="C21" s="18">
+        <v>206</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="C21" s="19">
         <v>0.1</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="C22" s="19">
+        <v>0.03</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="B22" s="16" t="s">
-        <v>201</v>
-      </c>
-      <c r="C22" s="18">
-        <v>0.03</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>192</v>
-      </c>
       <c r="E22" s="13" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="C23" s="10">
         <v>1200</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="15" t="s">
-        <v>205</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>206</v>
-      </c>
-      <c r="C24" s="17">
+        <v>213</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="C24" s="18">
         <v>200</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="C25" s="10">
         <v>25</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="15" t="s">
-        <v>211</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="C26" s="17">
+        <v>219</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="C26" s="18">
         <v>650</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C27" s="10">
         <v>50</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -3545,7 +3667,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3554,13 +3676,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
-        <v>216</v>
+      <c r="A1" s="16" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>14</v>
@@ -3572,13 +3694,13 @@
         <v>15</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>27</v>
@@ -3586,24 +3708,24 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="20">
         <v>36800</v>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="20">
         <v>1200</v>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="20">
         <f t="shared" ref="G4:G16" si="0">E4+F4</f>
         <v>38000</v>
       </c>
@@ -3611,24 +3733,24 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="20">
         <v>4100</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="20">
         <v>300</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="20">
         <f t="shared" si="0"/>
         <v>4400</v>
       </c>
@@ -3636,24 +3758,24 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="19">
+        <v>89</v>
+      </c>
+      <c r="E6" s="20">
         <v>150</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="20">
         <v>150</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="20">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
@@ -3661,24 +3783,24 @@
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E7" s="19">
+        <v>89</v>
+      </c>
+      <c r="E7" s="20">
         <v>3000</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="20">
         <v>0</v>
       </c>
-      <c r="G7" s="19">
+      <c r="G7" s="20">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
@@ -3686,24 +3808,24 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" s="19">
+        <v>89</v>
+      </c>
+      <c r="E8" s="20">
         <v>200</v>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="20">
         <v>0</v>
       </c>
-      <c r="G8" s="19">
+      <c r="G8" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
@@ -3711,24 +3833,24 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E9" s="19">
+        <v>89</v>
+      </c>
+      <c r="E9" s="20">
         <v>2600</v>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="20">
         <v>0</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="20">
         <f t="shared" si="0"/>
         <v>2600</v>
       </c>
@@ -3736,24 +3858,24 @@
     </row>
     <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="E10" s="19">
+        <v>249</v>
+      </c>
+      <c r="E10" s="20">
         <v>2200</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="20">
         <v>250</v>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="20">
         <f t="shared" si="0"/>
         <v>2450</v>
       </c>
@@ -3761,51 +3883,51 @@
     </row>
     <row r="11" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>243</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>244</v>
+        <v>251</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>252</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="E11" s="20">
+        <v>249</v>
+      </c>
+      <c r="E11" s="21">
         <v>3800</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="21">
         <v>200</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="21">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="20">
         <v>3000</v>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="20">
         <v>0</v>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="20">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
@@ -3813,24 +3935,24 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="20">
         <v>250</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="20">
         <v>0</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="20">
         <f t="shared" si="0"/>
         <v>250</v>
       </c>
@@ -3838,24 +3960,24 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E14" s="19">
+        <v>89</v>
+      </c>
+      <c r="E14" s="20">
         <v>250</v>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="20">
         <v>0</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="20">
         <f t="shared" si="0"/>
         <v>250</v>
       </c>
@@ -3863,24 +3985,24 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="20">
         <v>200</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="20">
         <v>0</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
@@ -3888,24 +4010,24 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="20">
         <v>110</v>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="20">
         <v>0</v>
       </c>
-      <c r="G16" s="19">
+      <c r="G16" s="20">
         <f t="shared" si="0"/>
         <v>110</v>
       </c>
@@ -3913,20 +4035,20 @@
     </row>
     <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="19">
+      <c r="G17" s="20">
         <f>0.3*CCement+1*CSand</f>
         <v>1620</v>
       </c>
@@ -3937,48 +4059,48 @@
         <v>12</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D20" s="7">
         <v>0</v>
@@ -3986,11 +4108,11 @@
       <c r="E20" s="7">
         <v>0.5</v>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="20">
         <f>CPlain</f>
         <v>2600</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="20">
         <f t="shared" ref="G20:G27" si="1">D20*(CRebar+CFixing)/1000</f>
         <v>0</v>
       </c>
@@ -3998,31 +4120,31 @@
         <f t="shared" ref="H20:H27" si="2">E20*CFormwork</f>
         <v>125</v>
       </c>
-      <c r="I20" s="19">
+      <c r="I20" s="20">
         <f t="shared" ref="I20:I27" si="3">CCasting</f>
         <v>250</v>
       </c>
-      <c r="J20" s="19">
+      <c r="J20" s="20">
         <f t="shared" ref="J20:J27" si="4">SUM(F20:I20)</f>
         <v>2975</v>
       </c>
-      <c r="K20" s="19">
+      <c r="K20" s="20">
         <v>25</v>
       </c>
-      <c r="L20" s="21">
+      <c r="L20" s="22">
         <f t="shared" ref="L20:L27" si="5">J20+K20</f>
         <v>3000</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D21" s="7">
         <v>100</v>
@@ -4030,11 +4152,11 @@
       <c r="E21" s="7">
         <v>1</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="20">
         <f t="shared" ref="F21:F27" si="6">CReadyMix+CPump</f>
         <v>3200</v>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="20">
         <f t="shared" si="1"/>
         <v>4100</v>
       </c>
@@ -4042,31 +4164,31 @@
         <f t="shared" si="2"/>
         <v>250</v>
       </c>
-      <c r="I21" s="19">
+      <c r="I21" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J21" s="19">
+      <c r="J21" s="20">
         <f t="shared" si="4"/>
         <v>7800</v>
       </c>
-      <c r="K21" s="19">
+      <c r="K21" s="20">
         <v>300</v>
       </c>
-      <c r="L21" s="21">
+      <c r="L21" s="22">
         <f t="shared" si="5"/>
         <v>8100</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D22" s="7">
         <v>50</v>
@@ -4074,11 +4196,11 @@
       <c r="E22" s="7">
         <v>0.3</v>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="20">
         <f t="shared" si="6"/>
         <v>3200</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="20">
         <f t="shared" si="1"/>
         <v>2050</v>
       </c>
@@ -4086,31 +4208,31 @@
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
-      <c r="I22" s="19">
+      <c r="I22" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="20">
         <f t="shared" si="4"/>
         <v>5575</v>
       </c>
-      <c r="K22" s="19">
+      <c r="K22" s="20">
         <v>-1075</v>
       </c>
-      <c r="L22" s="21">
+      <c r="L22" s="22">
         <f t="shared" si="5"/>
         <v>4500</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D23" s="7">
         <v>110</v>
@@ -4118,11 +4240,11 @@
       <c r="E23" s="7">
         <v>6.7</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="20">
         <f t="shared" si="6"/>
         <v>3200</v>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="20">
         <f t="shared" si="1"/>
         <v>4510</v>
       </c>
@@ -4130,31 +4252,31 @@
         <f t="shared" si="2"/>
         <v>1675</v>
       </c>
-      <c r="I23" s="19">
+      <c r="I23" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J23" s="19">
+      <c r="J23" s="20">
         <f t="shared" si="4"/>
         <v>9635</v>
       </c>
-      <c r="K23" s="19">
+      <c r="K23" s="20">
         <v>0</v>
       </c>
-      <c r="L23" s="21">
+      <c r="L23" s="22">
         <f t="shared" si="5"/>
         <v>9635</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D24" s="7">
         <v>170</v>
@@ -4162,11 +4284,11 @@
       <c r="E24" s="7">
         <v>11</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="20">
         <f t="shared" si="6"/>
         <v>3200</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="20">
         <f t="shared" si="1"/>
         <v>6970</v>
       </c>
@@ -4174,31 +4296,31 @@
         <f t="shared" si="2"/>
         <v>2750</v>
       </c>
-      <c r="I24" s="19">
+      <c r="I24" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J24" s="19">
+      <c r="J24" s="20">
         <f t="shared" si="4"/>
         <v>13170</v>
       </c>
-      <c r="K24" s="19">
+      <c r="K24" s="20">
         <v>-670</v>
       </c>
-      <c r="L24" s="21">
+      <c r="L24" s="22">
         <f t="shared" si="5"/>
         <v>12500</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D25" s="7">
         <v>130</v>
@@ -4206,11 +4328,11 @@
       <c r="E25" s="7">
         <v>4.5</v>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="20">
         <f t="shared" si="6"/>
         <v>3200</v>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="20">
         <f t="shared" si="1"/>
         <v>5330</v>
       </c>
@@ -4218,31 +4340,31 @@
         <f t="shared" si="2"/>
         <v>1125</v>
       </c>
-      <c r="I25" s="19">
+      <c r="I25" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J25" s="19">
+      <c r="J25" s="20">
         <f t="shared" si="4"/>
         <v>9905</v>
       </c>
-      <c r="K25" s="19">
+      <c r="K25" s="20">
         <v>-605</v>
       </c>
-      <c r="L25" s="21">
+      <c r="L25" s="22">
         <f t="shared" si="5"/>
         <v>9300</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D26" s="7">
         <v>110</v>
@@ -4250,11 +4372,11 @@
       <c r="E26" s="7">
         <v>5</v>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="20">
         <f t="shared" si="6"/>
         <v>3200</v>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="20">
         <f t="shared" si="1"/>
         <v>4510</v>
       </c>
@@ -4262,31 +4384,31 @@
         <f t="shared" si="2"/>
         <v>1250</v>
       </c>
-      <c r="I26" s="19">
+      <c r="I26" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J26" s="19">
+      <c r="J26" s="20">
         <f t="shared" si="4"/>
         <v>9210</v>
       </c>
-      <c r="K26" s="19">
+      <c r="K26" s="20">
         <v>290</v>
       </c>
-      <c r="L26" s="21">
+      <c r="L26" s="22">
         <f t="shared" si="5"/>
         <v>9500</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D27" s="7">
         <v>100</v>
@@ -4294,11 +4416,11 @@
       <c r="E27" s="7">
         <v>10</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="20">
         <f t="shared" si="6"/>
         <v>3200</v>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="20">
         <f t="shared" si="1"/>
         <v>4100</v>
       </c>
@@ -4306,18 +4428,18 @@
         <f t="shared" si="2"/>
         <v>2500</v>
       </c>
-      <c r="I27" s="19">
+      <c r="I27" s="20">
         <f t="shared" si="3"/>
         <v>250</v>
       </c>
-      <c r="J27" s="19">
+      <c r="J27" s="20">
         <f t="shared" si="4"/>
         <v>10050</v>
       </c>
-      <c r="K27" s="19">
+      <c r="K27" s="20">
         <v>-500</v>
       </c>
-      <c r="L27" s="21">
+      <c r="L27" s="22">
         <f t="shared" si="5"/>
         <v>9550</v>
       </c>
@@ -4327,192 +4449,192 @@
         <v>12</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="H29" s="5" t="s">
         <v>21</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D30" s="7">
         <v>110</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E30" s="23">
         <v>0.75</v>
       </c>
-      <c r="F30" s="23">
+      <c r="F30" s="24">
         <f>D30*(E30*CRedBrick+(1-E30)*CCementBrick)/1000</f>
         <v>312.125</v>
       </c>
-      <c r="G30" s="23">
+      <c r="G30" s="24">
         <f>0.05*CMortar</f>
         <v>81</v>
       </c>
-      <c r="H30" s="24">
+      <c r="H30" s="25">
         <f>CLabour25</f>
         <v>200</v>
       </c>
-      <c r="I30" s="23">
+      <c r="I30" s="24">
         <f>SUM(F30:H30)</f>
         <v>593.125</v>
       </c>
-      <c r="J30" s="23">
+      <c r="J30" s="24">
         <v>7</v>
       </c>
-      <c r="K30" s="25">
+      <c r="K30" s="26">
         <f>I30+J30</f>
         <v>600.125</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="7" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D31" s="7">
         <v>55</v>
       </c>
-      <c r="E31" s="22">
+      <c r="E31" s="23">
         <v>0.75</v>
       </c>
-      <c r="F31" s="23">
+      <c r="F31" s="24">
         <f>D31*(E31*CRedBrick+(1-E31)*CCementBrick)/1000</f>
         <v>156.0625</v>
       </c>
-      <c r="G31" s="23">
+      <c r="G31" s="24">
         <f>0.024*CMortar</f>
         <v>38.880000000000003</v>
       </c>
-      <c r="H31" s="24">
+      <c r="H31" s="25">
         <f>CLabour12</f>
         <v>110</v>
       </c>
-      <c r="I31" s="23">
+      <c r="I31" s="24">
         <f>SUM(F31:H31)</f>
         <v>304.9425</v>
       </c>
-      <c r="J31" s="23">
+      <c r="J31" s="24">
         <v>16</v>
       </c>
-      <c r="K31" s="25">
+      <c r="K31" s="26">
         <f>I31+J31</f>
         <v>320.9425</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D32" s="7">
         <v>110</v>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="23">
         <v>0</v>
       </c>
-      <c r="F32" s="23">
+      <c r="F32" s="24">
         <f>D32*(E32*CRedBrick+(1-E32)*CCementBrick)/1000</f>
         <v>440</v>
       </c>
-      <c r="G32" s="23">
+      <c r="G32" s="24">
         <f>0.05*CMortar</f>
         <v>81</v>
       </c>
-      <c r="H32" s="24">
+      <c r="H32" s="25">
         <f>CLabour25</f>
         <v>200</v>
       </c>
-      <c r="I32" s="23">
+      <c r="I32" s="24">
         <f>SUM(F32:H32)</f>
         <v>721</v>
       </c>
-      <c r="J32" s="23">
+      <c r="J32" s="24">
         <v>280</v>
       </c>
-      <c r="K32" s="25">
+      <c r="K32" s="26">
         <f>I32+J32</f>
         <v>1001</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D33" s="7">
         <v>55</v>
       </c>
-      <c r="E33" s="22">
+      <c r="E33" s="23">
         <v>0</v>
       </c>
-      <c r="F33" s="23">
+      <c r="F33" s="24">
         <f>D33*(E33*CRedBrick+(1-E33)*CCementBrick)/1000</f>
         <v>220</v>
       </c>
-      <c r="G33" s="23">
+      <c r="G33" s="24">
         <f>0.024*CMortar</f>
         <v>38.880000000000003</v>
       </c>
-      <c r="H33" s="24">
+      <c r="H33" s="25">
         <f>CLabour12</f>
         <v>110</v>
       </c>
-      <c r="I33" s="23">
+      <c r="I33" s="24">
         <f>SUM(F33:H33)</f>
         <v>368.88</v>
       </c>
-      <c r="J33" s="23">
+      <c r="J33" s="24">
         <v>131.19999999999999</v>
       </c>
-      <c r="K33" s="25">
+      <c r="K33" s="26">
         <f>I33+J33</f>
         <v>500.08</v>
       </c>
@@ -4531,228 +4653,246 @@
         <v>15</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E36" s="21">
+        <v>89</v>
+      </c>
+      <c r="E36" s="22">
         <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B37" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E37" s="21">
+      <c r="E37" s="22">
         <v>480</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E38" s="21">
+        <v>89</v>
+      </c>
+      <c r="E38" s="22">
         <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="7" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D39" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E39" s="21">
+      <c r="E39" s="22">
         <v>330</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D40" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E40" s="21">
+      <c r="E40" s="22">
         <v>350</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="7" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E41" s="21">
+      <c r="E41" s="22">
         <v>260</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A42" s="7" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E42" s="21">
+      <c r="E42" s="22">
         <v>250</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="7" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E43" s="21">
+      <c r="E43" s="22">
         <v>185</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="7" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D44" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E44" s="21">
+      <c r="E44" s="22">
         <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A45" s="7" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D45" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E45" s="21">
+      <c r="E45" s="22">
         <v>4200</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="7" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E46" s="21">
+      <c r="E46" s="22">
         <v>300</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="7" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E47" s="21">
+      <c r="E47" s="22">
         <v>2300</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="7" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="E48" s="21">
+        <v>164</v>
+      </c>
+      <c r="E48" s="22">
         <v>750000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E49" s="22">
+        <f>CRebar+CFixing</f>
+        <v>41000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rename to Construction Pricer; make all price sources anonymous (no reviewer, project or location)
</commit_message>
<xml_diff>
--- a/Price list - steel and metal works.xlsx
+++ b/Price list - steel and metal works.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Downloads\OnTap hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1940CF-538A-4A45-84C5-C8DE69C9D8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8161C40D-DC79-417B-8D65-40654BC0BE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
     <t>2. Their material prices are from the Ministry of Housing building materials price bulletin, August 2026 (including tax, excluding transport). The bulletin is in the sources folder.</t>
   </si>
   <si>
-    <t>3. Construction works (CW): prices from a reviewer's cost model, July 2026, delivered to site. The build-up is in the Construction sheet. 'Reviewer's adjustment' is the change he made by hand to the calculated price.</t>
+    <t>3. Construction works (CW): Egyptian market rates, July 2026, delivered to site, reviewed by a practising engineer. The build-up is in the Construction sheet. 'Market adjustment' is the hand correction applied to the calculated price.</t>
   </si>
   <si>
     <t>4. Yellow cells are estimates without a firm source. Please check them first.</t>
@@ -85,7 +85,7 @@
     <t>2. أسعار خاماتها من نشرة أسعار مواد البناء لوزارة الإسكان، أغسطس 2026 (شاملة الضرائب وغير شاملة النقل). النشرة موجودة في فولدر sources.</t>
   </si>
   <si>
-    <t>3. الأعمال الإنشائية (CW): الأسعار من نموذج تكلفة من مراجع، يوليو 2026، تسليم الموقع. تحليل السعر في شيت Construction، و'تعديل المراجع' هو الفرق الذي أضافه يدوياً على السعر المحسوب.</t>
+    <t>3. الأعمال الإنشائية (CW): أسعار السوق المصري، يوليو 2026، تسليم الموقع، مراجعة مهندس ممارس. تحليل السعر في شيت Construction، و'تعديل السوق' هو الفرق المضاف يدوياً على السعر المحسوب.</t>
   </si>
   <si>
     <t>4. الخلايا الصفراء تقديرات بدون مصدر مؤكد، برجاء مراجعتها أولاً.</t>
@@ -331,7 +331,7 @@
     <t>Construction</t>
   </si>
   <si>
-    <t>Reviewer's cost model, July 2026</t>
+    <t>Egyptian market cost model, July 2026 (reviewed by a practising engineer)</t>
   </si>
   <si>
     <t>CW-02</t>
@@ -562,7 +562,7 @@
     <t>Rebar, supply, cut, bend and fix</t>
   </si>
   <si>
-    <t>New item (Sep 2026): rebar + fixing from the reviewer's rates - please check</t>
+    <t>New item (Sep 2026): rebar + fixing from the model's rates - please check</t>
   </si>
   <si>
     <t>Cairo prices, including tax, excluding transport. Yellow = estimate, please check. No overhead or profit here.</t>
@@ -694,7 +694,7 @@
     <t>نقل للموقع</t>
   </si>
   <si>
-    <t>Reviewer's cost model: steel transport to site, July 2026</t>
+    <t>Egyptian market cost model, July 2026: steel transport to site</t>
   </si>
   <si>
     <t>Corrugated galvanized sheet 0.5 mm, supply</t>
@@ -730,7 +730,7 @@
     <t>ساندوتش بانل، تركيب</t>
   </si>
   <si>
-    <t>Reviewer's cost model, July 2026. Prices delivered to site. Unit price = calculated price + reviewer's adjustment (his hand change).</t>
+    <t>Egyptian market cost model, July 2026, reviewed by a practising engineer. Prices delivered to site. Unit price = calculated price + market adjustment (hand correction).</t>
   </si>
   <si>
     <t>Name</t>
@@ -817,7 +817,7 @@
     <t>طوب أسمنتي مصمت 25×12×6</t>
   </si>
   <si>
-    <t>His note says 1,400-1,800 per 1000 but he used 3,800 - ask him</t>
+    <t>Source note says 1,400-1,800 per 1000 but the model used 3,800 - please check</t>
   </si>
   <si>
     <t>CFixing</t>
@@ -901,7 +901,7 @@
     <t>Calculated price</t>
   </si>
   <si>
-    <t>Reviewer's adjustment</t>
+    <t>Market adjustment</t>
   </si>
   <si>
     <t>Unit price per m³</t>
@@ -2237,7 +2237,7 @@
       <c r="Q14" s="10"/>
       <c r="R14" s="9"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>86</v>
       </c>
@@ -2351,7 +2351,7 @@
       <c r="Q17" s="10"/>
       <c r="R17" s="9"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
         <v>98</v>
       </c>
@@ -2465,7 +2465,7 @@
       <c r="Q20" s="10"/>
       <c r="R20" s="9"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
         <v>107</v>
       </c>
@@ -2503,7 +2503,7 @@
       <c r="Q21" s="10"/>
       <c r="R21" s="9"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>110</v>
       </c>
@@ -2541,7 +2541,7 @@
       <c r="Q22" s="10"/>
       <c r="R22" s="9"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
         <v>113</v>
       </c>
@@ -2579,7 +2579,7 @@
       <c r="Q23" s="10"/>
       <c r="R23" s="9"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
         <v>116</v>
       </c>
@@ -2617,7 +2617,7 @@
       <c r="Q24" s="10"/>
       <c r="R24" s="9"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
         <v>119</v>
       </c>
@@ -2731,7 +2731,7 @@
       <c r="Q27" s="10"/>
       <c r="R27" s="9"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
         <v>128</v>
       </c>
@@ -2769,7 +2769,7 @@
       <c r="Q28" s="10"/>
       <c r="R28" s="9"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
         <v>131</v>
       </c>
@@ -2959,7 +2959,7 @@
       <c r="Q33" s="10"/>
       <c r="R33" s="9"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
         <v>146</v>
       </c>
@@ -2997,7 +2997,7 @@
       <c r="Q34" s="10"/>
       <c r="R34" s="9"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
         <v>149</v>
       </c>
@@ -3073,7 +3073,7 @@
       <c r="Q36" s="10"/>
       <c r="R36" s="9"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
         <v>155</v>
       </c>
@@ -3111,7 +3111,7 @@
       <c r="Q37" s="10"/>
       <c r="R37" s="9"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="7" t="s">
         <v>158</v>
       </c>
@@ -3187,7 +3187,7 @@
       <c r="Q39" s="10"/>
       <c r="R39" s="9"/>
     </row>
-    <row r="40" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A40" s="13" t="s">
         <v>165</v>
       </c>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="H10" s="9"/>
     </row>
-    <row r="11" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>250</v>
       </c>

</xml_diff>